<commit_message>
Bill number added in expense import
</commit_message>
<xml_diff>
--- a/uploads/expenses/file_sample/Sample_expense_item_en.xlsx
+++ b/uploads/expenses/file_sample/Sample_expense_item_en.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Vendors</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>Expense Date</t>
+  </si>
+  <si>
+    <t>Bill Number</t>
   </si>
 </sst>
 </file>
@@ -381,7 +384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -389,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="37.7109375" style="1" customWidth="1"/>
@@ -398,10 +401,11 @@
     <col min="4" max="4" width="33" style="3" customWidth="1"/>
     <col min="5" max="5" width="40.28515625" style="3" customWidth="1"/>
     <col min="6" max="6" width="24" style="3" customWidth="1"/>
-    <col min="7" max="16384" width="9.28515625" style="3"/>
+    <col min="7" max="7" width="21.140625" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="9.28515625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="50.25" customHeight="1">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="50.25" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -419,6 +423,9 @@
       </c>
       <c r="F1" s="4" t="s">
         <v>4</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>